<commit_message>
Novetats CIMA: 1 nous farmacos pendents de validacio
</commit_message>
<xml_diff>
--- a/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
+++ b/inhaladors_MPOC_ASMA_Avanzado_FINAL.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z179"/>
+  <dimension ref="A1:Z180"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="48.88" customWidth="1" style="28" min="1" max="1"/>
@@ -12901,6 +12901,81 @@
       </c>
       <c r="O179" s="29" t="inlineStr"/>
       <c r="P179" s="29" t="inlineStr"/>
+    </row>
+    <row r="180" ht="40" customHeight="1" s="28">
+      <c r="A180" s="29" t="inlineStr">
+        <is>
+          <t>LAMA</t>
+        </is>
+      </c>
+      <c r="B180" s="29" t="inlineStr">
+        <is>
+          <t>bromuro umeclidinio</t>
+        </is>
+      </c>
+      <c r="C180" s="29" t="inlineStr">
+        <is>
+          <t>INCRUSE ELLIPTA 55 MCG POLVO PARA INHALACION UNIDOSIS, 30 dosis</t>
+        </is>
+      </c>
+      <c r="D180" s="29" t="inlineStr">
+        <is>
+          <t>771325</t>
+        </is>
+      </c>
+      <c r="E180" s="29" t="inlineStr">
+        <is>
+          <t>INCRUSE ELLIPTA 55 MCG POLVO PARA INHALACION UNIDOSIS, 30 dosis</t>
+        </is>
+      </c>
+      <c r="F180" s="29" t="inlineStr">
+        <is>
+          <t>MPOC: 55 µg/24h
+D.màx: 55 µg/24h</t>
+        </is>
+      </c>
+      <c r="G180" s="29" t="inlineStr">
+        <is>
+          <t>IPS-multi</t>
+        </is>
+      </c>
+      <c r="H180" s="29" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="I180" s="29" t="inlineStr">
+        <is>
+          <t>&lt;50 l/m</t>
+        </is>
+      </c>
+      <c r="J180" s="29" t="inlineStr">
+        <is>
+          <t>Ràpida</t>
+        </is>
+      </c>
+      <c r="K180" s="29" t="inlineStr">
+        <is>
+          <t>https://scientiasalut.gencat.cat/handle/11351/11818</t>
+        </is>
+      </c>
+      <c r="L180" s="29" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="M180" s="29" t="inlineStr">
+        <is>
+          <t>https://cima.aemps.es/cima/publico/medicamento.html?nregistro=114922002IP2</t>
+        </is>
+      </c>
+      <c r="N180" s="29" t="inlineStr">
+        <is>
+          <t>NOU — PENDENT VALIDACIÓ CLÍNICA</t>
+        </is>
+      </c>
+      <c r="O180" s="29" t="inlineStr"/>
+      <c r="P180" s="29" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>